<commit_message>
2082/2083 pragati bibarann and krishi upaj provided and lamatol adhuro bhawan continue
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/2.0 कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१ sir.xlsx
+++ b/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/2.0 कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१ sir.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3E4839-0FA8-4570-9959-02B79B3EB120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="krishi thekka" sheetId="15" r:id="rId1"/>
@@ -34,7 +35,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'krishi thekka'!$A$1:$K$147</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'krishi thekka'!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -115,9 +116,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>F.Y.: 2082/2083</t>
   </si>
   <si>
     <t>Length (m)</t>
@@ -439,14 +437,17 @@
   <si>
     <t>-at paanipatti</t>
   </si>
+  <si>
+    <t>F.Y.:2082/2083</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -637,9 +638,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -655,14 +656,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -688,7 +689,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -721,7 +722,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -736,7 +737,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -775,11 +776,11 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -791,17 +792,29 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -814,32 +827,16 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -855,7 +852,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -949,7 +946,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1008,7 +1005,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1072,9 +1069,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1112,9 +1109,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1149,7 +1146,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1184,7 +1181,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1357,131 +1354,129 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K147"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" customWidth="1"/>
-    <col min="3" max="3" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+    <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="68" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-    </row>
-    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+    </row>
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="J3" s="70"/>
-      <c r="K3" s="70"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="70" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="70"/>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="70"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="70"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="70"/>
-    </row>
-    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="71" t="s">
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="71"/>
-      <c r="H5" s="71"/>
-      <c r="I5" s="71"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="71"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="66" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="60" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="67"/>
-      <c r="J6" s="67"/>
-      <c r="K6" s="67"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="60"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
+      <c r="H6" s="71" t="s">
+        <v>91</v>
+      </c>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="65"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
-    </row>
-    <row r="8" spans="1:11" s="10" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H7" s="70" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="70"/>
+      <c r="J7" s="70"/>
+    </row>
+    <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
         <v>5</v>
       </c>
@@ -1516,12 +1511,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="13" customFormat="1" ht="61.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" s="13" customFormat="1" ht="61.5" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>1</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="22"/>
@@ -1533,10 +1528,10 @@
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="B10" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="14">
         <v>2</v>
@@ -1558,10 +1553,10 @@
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
       <c r="B11" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="14">
         <v>2</v>
@@ -1583,10 +1578,10 @@
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
       <c r="B12" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" s="14">
         <v>1</v>
@@ -1609,7 +1604,7 @@
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="15"/>
       <c r="C13" s="14">
@@ -1633,10 +1628,10 @@
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="B14" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C14" s="14">
         <v>-1</v>
@@ -1657,7 +1652,7 @@
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
     </row>
-    <row r="15" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="17" t="s">
         <v>16</v>
@@ -1671,7 +1666,7 @@
         <v>33.017380559019209</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I15" s="2">
         <f>1.15*9949.51</f>
@@ -1683,7 +1678,7 @@
       </c>
       <c r="K15" s="19"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
@@ -1696,12 +1691,12 @@
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
     </row>
-    <row r="17" spans="1:11" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>2</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="22"/>
@@ -1713,10 +1708,10 @@
       <c r="J17" s="12"/>
       <c r="K17" s="12"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="B18" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" s="14">
         <v>1</v>
@@ -1739,10 +1734,10 @@
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C19" s="14">
         <v>-1</v>
@@ -1765,7 +1760,7 @@
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="B20" s="15"/>
       <c r="C20" s="14">
@@ -1789,7 +1784,7 @@
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
     </row>
-    <row r="21" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="17" t="s">
         <v>16</v>
@@ -1803,7 +1798,7 @@
         <v>10.044160865979912</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I21" s="2">
         <f>1.15*2808.56</f>
@@ -1815,7 +1810,7 @@
       </c>
       <c r="K21" s="19"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -1828,24 +1823,24 @@
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
     </row>
-    <row r="23" spans="1:11" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="23">
         <v>3</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C23" s="47" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E23" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="48" t="s">
         <v>36</v>
-      </c>
-      <c r="F23" s="48" t="s">
-        <v>37</v>
       </c>
       <c r="G23" s="26"/>
       <c r="H23" s="25"/>
@@ -1853,10 +1848,10 @@
       <c r="J23" s="21"/>
       <c r="K23" s="25"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
       <c r="B24" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C24" s="3">
         <f>6*TRUNC(3/0.42,0)</f>
@@ -1883,7 +1878,7 @@
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="15"/>
       <c r="C25" s="3">
@@ -1911,7 +1906,7 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
     </row>
-    <row r="26" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="17" t="s">
         <v>16</v>
@@ -1925,7 +1920,7 @@
         <v>2.5285877160305684E-2</v>
       </c>
       <c r="H26" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I26" s="2">
         <v>132360</v>
@@ -1936,7 +1931,7 @@
       </c>
       <c r="K26" s="19"/>
     </row>
-    <row r="27" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23"/>
       <c r="B27" s="24"/>
       <c r="C27" s="25"/>
@@ -1949,12 +1944,12 @@
       <c r="J27" s="21"/>
       <c r="K27" s="25"/>
     </row>
-    <row r="28" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="23">
         <v>4</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" s="25"/>
       <c r="D28" s="26"/>
@@ -1966,10 +1961,10 @@
       <c r="J28" s="21"/>
       <c r="K28" s="25"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
       <c r="B29" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" s="3">
         <v>6</v>
@@ -1991,7 +1986,7 @@
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
     </row>
-    <row r="30" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="17" t="s">
         <v>16</v>
@@ -2005,7 +2000,7 @@
         <v>6.4799999999999995</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I30" s="2">
         <v>922.71</v>
@@ -2016,7 +2011,7 @@
       </c>
       <c r="K30" s="19"/>
     </row>
-    <row r="31" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23"/>
       <c r="B31" s="24"/>
       <c r="C31" s="25"/>
@@ -2029,12 +2024,12 @@
       <c r="J31" s="21"/>
       <c r="K31" s="25"/>
     </row>
-    <row r="32" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="23">
         <v>5</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C32" s="25"/>
       <c r="D32" s="26"/>
@@ -2046,10 +2041,10 @@
       <c r="J32" s="21"/>
       <c r="K32" s="25"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
       <c r="B33" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C33" s="3">
         <v>6</v>
@@ -2073,7 +2068,7 @@
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
     </row>
-    <row r="34" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="17" t="s">
         <v>16</v>
@@ -2087,7 +2082,7 @@
         <v>0.48599999999999993</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I34" s="2">
         <v>13957.29</v>
@@ -2098,7 +2093,7 @@
       </c>
       <c r="K34" s="19"/>
     </row>
-    <row r="35" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="23"/>
       <c r="B35" s="24"/>
       <c r="C35" s="25"/>
@@ -2111,24 +2106,24 @@
       <c r="J35" s="21"/>
       <c r="K35" s="25"/>
     </row>
-    <row r="36" spans="1:11" ht="45" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
         <v>6</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C36" s="43" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="43" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E36" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="F36" s="43" t="s">
         <v>36</v>
-      </c>
-      <c r="F36" s="43" t="s">
-        <v>37</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="14"/>
@@ -2136,10 +2131,10 @@
       <c r="J36" s="14"/>
       <c r="K36" s="14"/>
     </row>
-    <row r="37" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
       <c r="B37" s="49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C37" s="57">
         <v>6</v>
@@ -2164,10 +2159,10 @@
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
     </row>
-    <row r="38" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11"/>
       <c r="B38" s="49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C38" s="58">
         <v>2</v>
@@ -2192,7 +2187,7 @@
       <c r="J38" s="14"/>
       <c r="K38" s="14"/>
     </row>
-    <row r="39" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="11"/>
       <c r="B39" s="27"/>
       <c r="C39" s="58">
@@ -2218,10 +2213,10 @@
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
     </row>
-    <row r="40" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="11"/>
       <c r="B40" s="49" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C40" s="57">
         <f>3*2</f>
@@ -2247,10 +2242,10 @@
       <c r="J40" s="14"/>
       <c r="K40" s="14"/>
     </row>
-    <row r="41" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="11"/>
       <c r="B41" s="49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C41" s="57">
         <v>3</v>
@@ -2275,10 +2270,10 @@
       <c r="J41" s="14"/>
       <c r="K41" s="14"/>
     </row>
-    <row r="42" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
       <c r="B42" s="49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C42" s="57">
         <f>3*2</f>
@@ -2304,7 +2299,7 @@
       <c r="J42" s="14"/>
       <c r="K42" s="14"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
       <c r="B43" s="49"/>
       <c r="C43" s="57">
@@ -2331,10 +2326,10 @@
       <c r="J43" s="14"/>
       <c r="K43" s="14"/>
     </row>
-    <row r="44" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
       <c r="B44" s="49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C44" s="57">
         <f>3*2</f>
@@ -2360,7 +2355,7 @@
       <c r="J44" s="14"/>
       <c r="K44" s="14"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
       <c r="B45" s="49"/>
       <c r="C45" s="57">
@@ -2387,10 +2382,10 @@
       <c r="J45" s="14"/>
       <c r="K45" s="14"/>
     </row>
-    <row r="46" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
       <c r="B46" s="49" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C46" s="57">
         <f>3*2</f>
@@ -2416,10 +2411,10 @@
       <c r="J46" s="14"/>
       <c r="K46" s="14"/>
     </row>
-    <row r="47" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="11"/>
       <c r="B47" s="49" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C47" s="26">
         <v>30</v>
@@ -2443,10 +2438,10 @@
       <c r="J47" s="14"/>
       <c r="K47" s="14"/>
     </row>
-    <row r="48" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="11"/>
       <c r="B48" s="44" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C48" s="3">
         <f>2*2</f>
@@ -2472,7 +2467,7 @@
       <c r="J48" s="14"/>
       <c r="K48" s="14"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
       <c r="B49" s="15"/>
       <c r="C49" s="3">
@@ -2499,7 +2494,7 @@
       <c r="J49" s="14"/>
       <c r="K49" s="14"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="11"/>
       <c r="B50" s="15"/>
       <c r="C50" s="3">
@@ -2526,7 +2521,7 @@
       <c r="J50" s="14"/>
       <c r="K50" s="14"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
       <c r="B51" s="15"/>
       <c r="C51" s="3">
@@ -2553,7 +2548,7 @@
       <c r="J51" s="14"/>
       <c r="K51" s="14"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="11"/>
       <c r="B52" s="15"/>
       <c r="C52" s="3">
@@ -2580,10 +2575,10 @@
       <c r="J52" s="14"/>
       <c r="K52" s="14"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="11"/>
       <c r="B53" s="56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -2595,10 +2590,10 @@
       <c r="J53" s="14"/>
       <c r="K53" s="14"/>
     </row>
-    <row r="54" spans="1:11" s="13" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="23"/>
       <c r="B54" s="52" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C54" s="53">
         <f>2*2</f>
@@ -2624,10 +2619,10 @@
       <c r="J54" s="55"/>
       <c r="K54" s="35"/>
     </row>
-    <row r="55" spans="1:11" s="13" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="23"/>
       <c r="B55" s="52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C55" s="53">
         <f>2*14</f>
@@ -2653,7 +2648,7 @@
       <c r="J55" s="55"/>
       <c r="K55" s="35"/>
     </row>
-    <row r="56" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="23"/>
       <c r="B56" s="52"/>
       <c r="C56" s="53">
@@ -2679,10 +2674,10 @@
       <c r="J56" s="55"/>
       <c r="K56" s="35"/>
     </row>
-    <row r="57" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="23"/>
       <c r="B57" s="52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C57" s="53">
         <f>14*2</f>
@@ -2707,7 +2702,7 @@
       <c r="J57" s="55"/>
       <c r="K57" s="35"/>
     </row>
-    <row r="58" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="23"/>
       <c r="B58" s="52"/>
       <c r="C58" s="53">
@@ -2733,10 +2728,10 @@
       <c r="J58" s="55"/>
       <c r="K58" s="35"/>
     </row>
-    <row r="59" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="23"/>
       <c r="B59" s="56" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C59" s="53"/>
       <c r="D59" s="54"/>
@@ -2748,10 +2743,10 @@
       <c r="J59" s="55"/>
       <c r="K59" s="35"/>
     </row>
-    <row r="60" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="11"/>
       <c r="B60" s="49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C60" s="57">
         <v>5</v>
@@ -2775,7 +2770,7 @@
       <c r="J60" s="14"/>
       <c r="K60" s="14"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="11"/>
       <c r="B61" s="49"/>
       <c r="C61" s="57">
@@ -2801,7 +2796,7 @@
       <c r="J61" s="14"/>
       <c r="K61" s="14"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="11"/>
       <c r="B62" s="49"/>
       <c r="C62" s="57">
@@ -2827,7 +2822,7 @@
       <c r="J62" s="14"/>
       <c r="K62" s="14"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="11"/>
       <c r="B63" s="49"/>
       <c r="C63" s="57">
@@ -2853,10 +2848,10 @@
       <c r="J63" s="14"/>
       <c r="K63" s="14"/>
     </row>
-    <row r="64" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="11"/>
       <c r="B64" s="49" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C64" s="57">
         <f>C62*2</f>
@@ -2882,7 +2877,7 @@
       <c r="J64" s="14"/>
       <c r="K64" s="14"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="11"/>
       <c r="B65" s="49"/>
       <c r="C65" s="57">
@@ -2909,7 +2904,7 @@
       <c r="J65" s="14"/>
       <c r="K65" s="14"/>
     </row>
-    <row r="66" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="16"/>
       <c r="B66" s="17" t="s">
         <v>16</v>
@@ -2923,7 +2918,7 @@
         <v>1297.1697458092044</v>
       </c>
       <c r="H66" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I66" s="2">
         <f>1.15*182.51</f>
@@ -2935,7 +2930,7 @@
       </c>
       <c r="K66" s="19"/>
     </row>
-    <row r="67" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="16"/>
       <c r="B67" s="17"/>
       <c r="C67" s="18"/>
@@ -2948,12 +2943,12 @@
       <c r="J67" s="21"/>
       <c r="K67" s="19"/>
     </row>
-    <row r="68" spans="1:11" s="10" customFormat="1" ht="43.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="23">
         <v>7</v>
       </c>
       <c r="B68" s="27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C68" s="27"/>
       <c r="D68" s="26"/>
@@ -2965,10 +2960,10 @@
       <c r="J68" s="21"/>
       <c r="K68" s="25"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="11"/>
       <c r="B69" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C69" s="3">
         <v>2</v>
@@ -2991,7 +2986,7 @@
       <c r="J69" s="14"/>
       <c r="K69" s="14"/>
     </row>
-    <row r="70" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="16"/>
       <c r="B70" s="17" t="s">
         <v>16</v>
@@ -3005,7 +3000,7 @@
         <v>64.241756194007564</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I70" s="2">
         <v>1890.42</v>
@@ -3016,7 +3011,7 @@
       </c>
       <c r="K70" s="19"/>
     </row>
-    <row r="71" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="23"/>
       <c r="B71" s="24"/>
       <c r="C71" s="25"/>
@@ -3029,12 +3024,12 @@
       <c r="J71" s="21"/>
       <c r="K71" s="25"/>
     </row>
-    <row r="72" spans="1:11" s="10" customFormat="1" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" s="10" customFormat="1" ht="69" x14ac:dyDescent="0.25">
       <c r="A72" s="23">
         <v>8</v>
       </c>
       <c r="B72" s="27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C72" s="27"/>
       <c r="D72" s="26"/>
@@ -3046,7 +3041,7 @@
       <c r="J72" s="21"/>
       <c r="K72" s="25"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="11"/>
       <c r="B73" s="15" t="str">
         <f>B69</f>
@@ -3070,7 +3065,7 @@
       <c r="J73" s="14"/>
       <c r="K73" s="14"/>
     </row>
-    <row r="74" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="16"/>
       <c r="B74" s="17" t="s">
         <v>16</v>
@@ -3084,7 +3079,7 @@
         <v>10.362694300518134</v>
       </c>
       <c r="H74" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I74" s="2">
         <v>2771.25</v>
@@ -3095,7 +3090,7 @@
       </c>
       <c r="K74" s="19"/>
     </row>
-    <row r="75" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="23"/>
       <c r="B75" s="24"/>
       <c r="C75" s="25"/>
@@ -3108,12 +3103,12 @@
       <c r="J75" s="21"/>
       <c r="K75" s="25"/>
     </row>
-    <row r="76" spans="1:11" s="10" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" s="10" customFormat="1" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="23">
         <v>9</v>
       </c>
       <c r="B76" s="50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C76" s="50"/>
       <c r="D76" s="26"/>
@@ -3125,10 +3120,10 @@
       <c r="J76" s="21"/>
       <c r="K76" s="25"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="11"/>
       <c r="B77" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C77" s="3">
         <v>1</v>
@@ -3151,7 +3146,7 @@
       <c r="J77" s="14"/>
       <c r="K77" s="14"/>
     </row>
-    <row r="78" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="16"/>
       <c r="B78" s="17" t="s">
         <v>16</v>
@@ -3165,7 +3160,7 @@
         <v>35.740956237556269</v>
       </c>
       <c r="H78" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I78" s="2">
         <v>1422.19</v>
@@ -3176,7 +3171,7 @@
       </c>
       <c r="K78" s="19"/>
     </row>
-    <row r="79" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="23"/>
       <c r="B79" s="24"/>
       <c r="C79" s="25"/>
@@ -3189,12 +3184,12 @@
       <c r="J79" s="21"/>
       <c r="K79" s="25"/>
     </row>
-    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="11">
         <v>10</v>
       </c>
       <c r="B80" s="27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C80" s="14"/>
       <c r="D80" s="14"/>
@@ -3206,10 +3201,10 @@
       <c r="J80" s="14"/>
       <c r="K80" s="14"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="11"/>
       <c r="B81" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C81" s="3">
         <v>2</v>
@@ -3234,7 +3229,7 @@
       <c r="J81" s="14"/>
       <c r="K81" s="14"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="11"/>
       <c r="B82" s="15"/>
       <c r="C82" s="3">
@@ -3261,7 +3256,7 @@
       <c r="J82" s="14"/>
       <c r="K82" s="14"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="11"/>
       <c r="B83" s="15"/>
       <c r="C83" s="3">
@@ -3286,7 +3281,7 @@
       <c r="J83" s="14"/>
       <c r="K83" s="14"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="11"/>
       <c r="B84" s="15"/>
       <c r="C84" s="3">
@@ -3313,10 +3308,10 @@
       <c r="J84" s="14"/>
       <c r="K84" s="14"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="11"/>
       <c r="B85" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C85" s="3">
         <v>-2</v>
@@ -3339,7 +3334,7 @@
       <c r="J85" s="14"/>
       <c r="K85" s="14"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="11"/>
       <c r="B86" s="15"/>
       <c r="C86" s="3">
@@ -3363,10 +3358,10 @@
       <c r="J86" s="14"/>
       <c r="K86" s="14"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="11"/>
       <c r="B87" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C87" s="3">
         <v>-1</v>
@@ -3389,7 +3384,7 @@
       <c r="J87" s="14"/>
       <c r="K87" s="14"/>
     </row>
-    <row r="88" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="16"/>
       <c r="B88" s="17" t="s">
         <v>16</v>
@@ -3403,7 +3398,7 @@
         <v>13.473939774459005</v>
       </c>
       <c r="H88" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I88" s="2">
         <f>1.15*14491.84</f>
@@ -3415,7 +3410,7 @@
       </c>
       <c r="K88" s="19"/>
     </row>
-    <row r="89" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="23"/>
       <c r="B89" s="24"/>
       <c r="C89" s="25"/>
@@ -3428,12 +3423,12 @@
       <c r="J89" s="21"/>
       <c r="K89" s="25"/>
     </row>
-    <row r="90" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="11">
         <v>11</v>
       </c>
       <c r="B90" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C90" s="14"/>
       <c r="D90" s="14"/>
@@ -3445,10 +3440,10 @@
       <c r="J90" s="14"/>
       <c r="K90" s="14"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="11"/>
       <c r="B91" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C91" s="51">
         <v>1</v>
@@ -3471,7 +3466,7 @@
       <c r="J91" s="14"/>
       <c r="K91" s="14"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="11"/>
       <c r="B92" s="15" t="str">
         <f>B85</f>
@@ -3499,7 +3494,7 @@
       <c r="J92" s="14"/>
       <c r="K92" s="14"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="11"/>
       <c r="B93" s="15"/>
       <c r="C93" s="51">
@@ -3524,7 +3519,7 @@
       <c r="J93" s="14"/>
       <c r="K93" s="14"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="11"/>
       <c r="B94" s="15" t="str">
         <f>B87</f>
@@ -3552,10 +3547,10 @@
       <c r="J94" s="14"/>
       <c r="K94" s="14"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="11"/>
       <c r="B95" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C95" s="51">
         <v>1</v>
@@ -3578,7 +3573,7 @@
       <c r="J95" s="14"/>
       <c r="K95" s="14"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="11"/>
       <c r="B96" s="15" t="str">
         <f>B85</f>
@@ -3606,7 +3601,7 @@
       <c r="J96" s="14"/>
       <c r="K96" s="14"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="11"/>
       <c r="B97" s="15"/>
       <c r="C97" s="51">
@@ -3631,7 +3626,7 @@
       <c r="J97" s="14"/>
       <c r="K97" s="14"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="11"/>
       <c r="B98" s="15" t="str">
         <f>B87</f>
@@ -3659,10 +3654,10 @@
       <c r="J98" s="14"/>
       <c r="K98" s="14"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="11"/>
       <c r="B99" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C99" s="51">
         <v>-1</v>
@@ -3684,7 +3679,7 @@
       <c r="J99" s="14"/>
       <c r="K99" s="14"/>
     </row>
-    <row r="100" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="16"/>
       <c r="B100" s="17" t="s">
         <v>16</v>
@@ -3698,7 +3693,7 @@
         <v>104.25673516513439</v>
       </c>
       <c r="H100" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I100" s="2">
         <f>1.15*415.5</f>
@@ -3710,7 +3705,7 @@
       </c>
       <c r="K100" s="19"/>
     </row>
-    <row r="101" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="23"/>
       <c r="B101" s="24"/>
       <c r="C101" s="25"/>
@@ -3723,12 +3718,12 @@
       <c r="J101" s="21"/>
       <c r="K101" s="25"/>
     </row>
-    <row r="102" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="11">
         <v>12</v>
       </c>
       <c r="B102" s="27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C102" s="14"/>
       <c r="D102" s="14"/>
@@ -3740,10 +3735,10 @@
       <c r="J102" s="14"/>
       <c r="K102" s="14"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="11"/>
       <c r="B103" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C103" s="3">
         <v>1</v>
@@ -3763,10 +3758,10 @@
       <c r="J103" s="14"/>
       <c r="K103" s="14"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" s="11"/>
       <c r="B104" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C104" s="3">
         <v>1</v>
@@ -3789,10 +3784,10 @@
       <c r="J104" s="14"/>
       <c r="K104" s="14"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="11"/>
       <c r="B105" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C105" s="3">
         <v>-2</v>
@@ -3813,7 +3808,7 @@
       <c r="J105" s="14"/>
       <c r="K105" s="14"/>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="11"/>
       <c r="B106" s="15"/>
       <c r="C106" s="3">
@@ -3835,10 +3830,10 @@
       <c r="J106" s="14"/>
       <c r="K106" s="14"/>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="11"/>
       <c r="B107" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C107" s="3">
         <v>-1</v>
@@ -3860,7 +3855,7 @@
       <c r="J107" s="14"/>
       <c r="K107" s="14"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="11"/>
       <c r="B108" s="15"/>
       <c r="C108" s="3">
@@ -3883,10 +3878,10 @@
       <c r="J108" s="14"/>
       <c r="K108" s="14"/>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" s="11"/>
       <c r="B109" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C109" s="3">
         <v>2</v>
@@ -3908,10 +3903,10 @@
       <c r="J109" s="14"/>
       <c r="K109" s="14"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="11"/>
       <c r="B110" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C110" s="3">
         <v>-1</v>
@@ -3932,10 +3927,10 @@
       <c r="J110" s="14"/>
       <c r="K110" s="14"/>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" s="11"/>
       <c r="B111" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C111" s="3">
         <v>1</v>
@@ -3957,7 +3952,7 @@
       <c r="J111" s="14"/>
       <c r="K111" s="14"/>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="11"/>
       <c r="B112" s="15"/>
       <c r="C112" s="3">
@@ -3980,7 +3975,7 @@
       <c r="J112" s="14"/>
       <c r="K112" s="14"/>
     </row>
-    <row r="113" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="16"/>
       <c r="B113" s="17" t="s">
         <v>16</v>
@@ -3994,7 +3989,7 @@
         <v>141.11398631820401</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I113" s="2">
         <f>1.15*253.8</f>
@@ -4006,7 +4001,7 @@
       </c>
       <c r="K113" s="19"/>
     </row>
-    <row r="114" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="23"/>
       <c r="B114" s="24"/>
       <c r="C114" s="25"/>
@@ -4019,12 +4014,12 @@
       <c r="J114" s="21"/>
       <c r="K114" s="25"/>
     </row>
-    <row r="115" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A115" s="11">
         <v>13</v>
       </c>
       <c r="B115" s="27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C115" s="14"/>
       <c r="D115" s="14"/>
@@ -4036,10 +4031,10 @@
       <c r="J115" s="14"/>
       <c r="K115" s="14"/>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="11"/>
       <c r="B116" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C116" s="3">
         <v>1</v>
@@ -4059,10 +4054,10 @@
       <c r="J116" s="14"/>
       <c r="K116" s="14"/>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="11"/>
       <c r="B117" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C117" s="3">
         <v>1</v>
@@ -4085,10 +4080,10 @@
       <c r="J117" s="14"/>
       <c r="K117" s="14"/>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="11"/>
       <c r="B118" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C118" s="3">
         <v>-2</v>
@@ -4109,7 +4104,7 @@
       <c r="J118" s="14"/>
       <c r="K118" s="14"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="11"/>
       <c r="B119" s="15"/>
       <c r="C119" s="3">
@@ -4131,10 +4126,10 @@
       <c r="J119" s="14"/>
       <c r="K119" s="14"/>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="11"/>
       <c r="B120" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C120" s="3">
         <v>-1</v>
@@ -4156,7 +4151,7 @@
       <c r="J120" s="14"/>
       <c r="K120" s="14"/>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="11"/>
       <c r="B121" s="15"/>
       <c r="C121" s="3">
@@ -4179,7 +4174,7 @@
       <c r="J121" s="14"/>
       <c r="K121" s="14"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="11"/>
       <c r="B122" s="15"/>
       <c r="C122" s="3">
@@ -4201,10 +4196,10 @@
       <c r="J122" s="14"/>
       <c r="K122" s="14"/>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="11"/>
       <c r="B123" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C123" s="3">
         <v>2</v>
@@ -4226,10 +4221,10 @@
       <c r="J123" s="14"/>
       <c r="K123" s="14"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="11"/>
       <c r="B124" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C124" s="3">
         <v>-1</v>
@@ -4250,7 +4245,7 @@
       <c r="J124" s="14"/>
       <c r="K124" s="14"/>
     </row>
-    <row r="125" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="16"/>
       <c r="B125" s="17" t="s">
         <v>16</v>
@@ -4264,7 +4259,7 @@
         <v>126.99591726992787</v>
       </c>
       <c r="H125" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I125" s="2">
         <v>214.41</v>
@@ -4275,7 +4270,7 @@
       </c>
       <c r="K125" s="19"/>
     </row>
-    <row r="126" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="23"/>
       <c r="B126" s="24"/>
       <c r="C126" s="25"/>
@@ -4288,12 +4283,12 @@
       <c r="J126" s="21"/>
       <c r="K126" s="25"/>
     </row>
-    <row r="127" spans="1:11" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" s="10" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A127" s="23">
         <v>14</v>
       </c>
       <c r="B127" s="50" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C127" s="50"/>
       <c r="D127" s="26"/>
@@ -4305,10 +4300,10 @@
       <c r="J127" s="21"/>
       <c r="K127" s="25"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="11"/>
       <c r="B128" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C128" s="3">
         <v>1</v>
@@ -4329,7 +4324,7 @@
       <c r="J128" s="14"/>
       <c r="K128" s="14"/>
     </row>
-    <row r="129" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="16"/>
       <c r="B129" s="17" t="s">
         <v>16</v>
@@ -4343,7 +4338,7 @@
         <v>2.52</v>
       </c>
       <c r="H129" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I129" s="2">
         <v>10055.6</v>
@@ -4354,7 +4349,7 @@
       </c>
       <c r="K129" s="19"/>
     </row>
-    <row r="130" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="23"/>
       <c r="B130" s="24"/>
       <c r="C130" s="25"/>
@@ -4367,12 +4362,12 @@
       <c r="J130" s="21"/>
       <c r="K130" s="25"/>
     </row>
-    <row r="131" spans="1:11" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" s="10" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A131" s="23">
         <v>15</v>
       </c>
       <c r="B131" s="50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C131" s="50"/>
       <c r="D131" s="26"/>
@@ -4384,10 +4379,10 @@
       <c r="J131" s="21"/>
       <c r="K131" s="25"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" s="11"/>
       <c r="B132" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C132" s="3">
         <v>2</v>
@@ -4408,7 +4403,7 @@
       <c r="J132" s="14"/>
       <c r="K132" s="14"/>
     </row>
-    <row r="133" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="16"/>
       <c r="B133" s="17" t="s">
         <v>16</v>
@@ -4422,7 +4417,7 @@
         <v>4.32</v>
       </c>
       <c r="H133" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I133" s="2">
         <v>8046.55</v>
@@ -4433,7 +4428,7 @@
       </c>
       <c r="K133" s="19"/>
     </row>
-    <row r="134" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="23"/>
       <c r="B134" s="24"/>
       <c r="C134" s="25"/>
@@ -4446,12 +4441,12 @@
       <c r="J134" s="21"/>
       <c r="K134" s="25"/>
     </row>
-    <row r="135" spans="1:11" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" s="10" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A135" s="23">
         <v>16</v>
       </c>
       <c r="B135" s="50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C135" s="50"/>
       <c r="D135" s="26"/>
@@ -4463,10 +4458,10 @@
       <c r="J135" s="21"/>
       <c r="K135" s="25"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" s="11"/>
       <c r="B136" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C136" s="3">
         <v>2</v>
@@ -4487,7 +4482,7 @@
       <c r="J136" s="14"/>
       <c r="K136" s="14"/>
     </row>
-    <row r="137" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="16"/>
       <c r="B137" s="17" t="s">
         <v>16</v>
@@ -4501,7 +4496,7 @@
         <v>2.88</v>
       </c>
       <c r="H137" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I137" s="2">
         <v>8046.55</v>
@@ -4512,7 +4507,7 @@
       </c>
       <c r="K137" s="19"/>
     </row>
-    <row r="138" spans="1:11" s="10" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:11" s="10" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="23"/>
       <c r="B138" s="24"/>
       <c r="C138" s="25"/>
@@ -4525,12 +4520,12 @@
       <c r="J138" s="21"/>
       <c r="K138" s="25"/>
     </row>
-    <row r="139" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="16">
         <v>17</v>
       </c>
       <c r="B139" s="45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C139" s="18">
         <v>1</v>
@@ -4543,7 +4538,7 @@
         <v>1</v>
       </c>
       <c r="H139" s="20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I139" s="2">
         <v>5000</v>
@@ -4554,7 +4549,7 @@
       </c>
       <c r="K139" s="19"/>
     </row>
-    <row r="140" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="23"/>
       <c r="B140" s="24"/>
       <c r="C140" s="25"/>
@@ -4567,7 +4562,7 @@
       <c r="J140" s="21"/>
       <c r="K140" s="25"/>
     </row>
-    <row r="141" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="16">
         <v>18</v>
       </c>
@@ -4596,7 +4591,7 @@
       </c>
       <c r="K141" s="19"/>
     </row>
-    <row r="142" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="16"/>
       <c r="B142" s="29"/>
       <c r="C142" s="18"/>
@@ -4609,7 +4604,7 @@
       <c r="J142" s="21"/>
       <c r="K142" s="19"/>
     </row>
-    <row r="143" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="42"/>
       <c r="B143" s="30" t="s">
         <v>20</v>
@@ -4627,19 +4622,19 @@
       </c>
       <c r="K143" s="33"/>
     </row>
-    <row r="144" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="40"/>
     </row>
-    <row r="145" spans="1:10" s="40" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="34"/>
       <c r="B145" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="C145" s="62">
+      <c r="C145" s="66">
         <f>J143</f>
         <v>1331142.8392085307</v>
       </c>
-      <c r="D145" s="63"/>
+      <c r="D145" s="67"/>
       <c r="E145" s="34"/>
       <c r="F145" s="36"/>
       <c r="G145" s="34"/>
@@ -4647,45 +4642,43 @@
       <c r="I145" s="38"/>
       <c r="J145" s="39"/>
     </row>
-    <row r="146" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="40"/>
       <c r="B146" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="C146" s="64">
+        <v>45</v>
+      </c>
+      <c r="C146" s="68">
         <f>0.13*C145</f>
         <v>173048.56909710899</v>
       </c>
-      <c r="D146" s="65"/>
-    </row>
-    <row r="147" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D146" s="69"/>
+    </row>
+    <row r="147" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="40"/>
       <c r="B147" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="C147" s="64">
+        <v>46</v>
+      </c>
+      <c r="C147" s="68">
         <f>SUM(C145:D146)</f>
         <v>1504191.4083056396</v>
       </c>
-      <c r="D147" s="65"/>
+      <c r="D147" s="69"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="10">
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="C145:D145"/>
+    <mergeCell ref="C146:D146"/>
+    <mergeCell ref="C147:D147"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C145:D145"/>
-    <mergeCell ref="C146:D146"/>
-    <mergeCell ref="C147:D147"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="80" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
krishi upaj print to oda adhaxya and rimal pandhero gairabaari sadak estimate and asked to  nabin sir and gh section remaining
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/2.0 कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१ sir.xlsx
+++ b/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/2.0 कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१ sir.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3E4839-0FA8-4570-9959-02B79B3EB120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC7D7D3-D3AA-4C8E-87BC-8A1238DB4590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -793,27 +793,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -827,8 +811,24 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1360,121 +1360,121 @@
   <cols>
     <col min="1" max="1" width="4.7109375" style="13" customWidth="1"/>
     <col min="2" max="2" width="30.85546875" customWidth="1"/>
-    <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.42578125" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" customWidth="1"/>
     <col min="6" max="6" width="7.28515625" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" customWidth="1"/>
     <col min="10" max="10" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
+      <c r="B5" s="70"/>
+      <c r="C5" s="70"/>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="70"/>
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="70"/>
+      <c r="K5" s="70"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="71" t="s">
+      <c r="H6" s="60" t="s">
         <v>91</v>
       </c>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="65" t="s">
+      <c r="A7" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="65"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="70" t="s">
+      <c r="H7" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="70"/>
-      <c r="J7" s="70"/>
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
@@ -1533,7 +1533,7 @@
       <c r="B10" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="51">
         <v>2</v>
       </c>
       <c r="D10" s="3">
@@ -1558,7 +1558,7 @@
       <c r="B11" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="51">
         <v>2</v>
       </c>
       <c r="D11" s="3">
@@ -1583,7 +1583,7 @@
       <c r="B12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="51">
         <v>1</v>
       </c>
       <c r="D12" s="3">
@@ -1607,7 +1607,7 @@
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="15"/>
-      <c r="C13" s="14">
+      <c r="C13" s="51">
         <v>1</v>
       </c>
       <c r="D13" s="3">
@@ -1633,7 +1633,7 @@
       <c r="B14" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="51">
         <v>-1</v>
       </c>
       <c r="D14" s="3">
@@ -1713,7 +1713,7 @@
       <c r="B18" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="51">
         <v>1</v>
       </c>
       <c r="D18" s="3">
@@ -1739,7 +1739,7 @@
       <c r="B19" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="51">
         <v>-1</v>
       </c>
       <c r="D19" s="3">
@@ -1763,7 +1763,7 @@
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="B20" s="15"/>
-      <c r="C20" s="14">
+      <c r="C20" s="51">
         <v>-1</v>
       </c>
       <c r="D20" s="3">
@@ -1853,7 +1853,7 @@
       <c r="B24" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="51">
         <f>6*TRUNC(3/0.42,0)</f>
         <v>42</v>
       </c>
@@ -1881,7 +1881,7 @@
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="15"/>
-      <c r="C25" s="3">
+      <c r="C25" s="51">
         <f>C24</f>
         <v>42</v>
       </c>
@@ -1922,7 +1922,7 @@
       <c r="H26" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="71">
         <v>132360</v>
       </c>
       <c r="J26" s="21">
@@ -1966,7 +1966,7 @@
       <c r="B29" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29" s="51">
         <v>6</v>
       </c>
       <c r="D29" s="3">
@@ -2046,7 +2046,7 @@
       <c r="B33" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="51">
         <v>6</v>
       </c>
       <c r="D33" s="3">
@@ -2164,10 +2164,10 @@
       <c r="B38" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="58">
+      <c r="C38" s="51">
         <v>2</v>
       </c>
-      <c r="D38" s="59">
+      <c r="D38" s="58">
         <f>14.25/3.281</f>
         <v>4.3431880524230415</v>
       </c>
@@ -2190,10 +2190,10 @@
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="11"/>
       <c r="B39" s="27"/>
-      <c r="C39" s="58">
+      <c r="C39" s="51">
         <v>3</v>
       </c>
-      <c r="D39" s="59">
+      <c r="D39" s="58">
         <f>(14.25+2.5+2)/3.281</f>
         <v>5.7147211216092648</v>
       </c>
@@ -2416,7 +2416,7 @@
       <c r="B47" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="C47" s="26">
+      <c r="C47" s="51">
         <v>30</v>
       </c>
       <c r="D47" s="26">
@@ -2443,7 +2443,7 @@
       <c r="B48" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="C48" s="3">
+      <c r="C48" s="51">
         <f>2*2</f>
         <v>4</v>
       </c>
@@ -2470,7 +2470,7 @@
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
       <c r="B49" s="15"/>
-      <c r="C49" s="3">
+      <c r="C49" s="51">
         <f>2*2</f>
         <v>4</v>
       </c>
@@ -2497,7 +2497,7 @@
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="11"/>
       <c r="B50" s="15"/>
-      <c r="C50" s="3">
+      <c r="C50" s="51">
         <f>5*2</f>
         <v>10</v>
       </c>
@@ -2524,7 +2524,7 @@
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
       <c r="B51" s="15"/>
-      <c r="C51" s="3">
+      <c r="C51" s="51">
         <f>1*2</f>
         <v>2</v>
       </c>
@@ -2551,7 +2551,7 @@
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="11"/>
       <c r="B52" s="15"/>
-      <c r="C52" s="3">
+      <c r="C52" s="51">
         <f>2*2</f>
         <v>4</v>
       </c>
@@ -2965,7 +2965,7 @@
       <c r="B69" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C69" s="3">
+      <c r="C69" s="51">
         <v>2</v>
       </c>
       <c r="D69" s="3">
@@ -3047,7 +3047,7 @@
         <f>B69</f>
         <v>-for roof</v>
       </c>
-      <c r="C73" s="3">
+      <c r="C73" s="51">
         <v>1</v>
       </c>
       <c r="D73" s="3">
@@ -3125,7 +3125,7 @@
       <c r="B77" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C77" s="3">
+      <c r="C77" s="51">
         <v>1</v>
       </c>
       <c r="D77" s="3">
@@ -3206,7 +3206,7 @@
       <c r="B81" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="C81" s="3">
+      <c r="C81" s="51">
         <v>2</v>
       </c>
       <c r="D81" s="3">
@@ -3232,7 +3232,7 @@
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="11"/>
       <c r="B82" s="15"/>
-      <c r="C82" s="3">
+      <c r="C82" s="51">
         <f>C81</f>
         <v>2</v>
       </c>
@@ -3259,7 +3259,7 @@
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="11"/>
       <c r="B83" s="15"/>
-      <c r="C83" s="3">
+      <c r="C83" s="51">
         <v>4</v>
       </c>
       <c r="D83" s="3">
@@ -3284,7 +3284,7 @@
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="11"/>
       <c r="B84" s="15"/>
-      <c r="C84" s="3">
+      <c r="C84" s="51">
         <f>C83</f>
         <v>4</v>
       </c>
@@ -3313,7 +3313,7 @@
       <c r="B85" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="C85" s="3">
+      <c r="C85" s="51">
         <v>-2</v>
       </c>
       <c r="D85" s="3">
@@ -3337,7 +3337,7 @@
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="11"/>
       <c r="B86" s="15"/>
-      <c r="C86" s="3">
+      <c r="C86" s="51">
         <v>-2</v>
       </c>
       <c r="D86" s="3">
@@ -3363,7 +3363,7 @@
       <c r="B87" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C87" s="3">
+      <c r="C87" s="51">
         <v>-1</v>
       </c>
       <c r="D87" s="3">
@@ -3740,7 +3740,7 @@
       <c r="B103" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="C103" s="3">
+      <c r="C103" s="51">
         <v>1</v>
       </c>
       <c r="D103" s="3">
@@ -3763,7 +3763,7 @@
       <c r="B104" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C104" s="3">
+      <c r="C104" s="51">
         <v>1</v>
       </c>
       <c r="D104" s="3">
@@ -3789,7 +3789,7 @@
       <c r="B105" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="C105" s="3">
+      <c r="C105" s="51">
         <v>-2</v>
       </c>
       <c r="D105" s="3">
@@ -3811,7 +3811,7 @@
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="11"/>
       <c r="B106" s="15"/>
-      <c r="C106" s="3">
+      <c r="C106" s="51">
         <v>-1</v>
       </c>
       <c r="D106" s="3">
@@ -3835,7 +3835,7 @@
       <c r="B107" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C107" s="3">
+      <c r="C107" s="51">
         <v>-1</v>
       </c>
       <c r="D107" s="3">
@@ -3858,7 +3858,7 @@
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="11"/>
       <c r="B108" s="15"/>
-      <c r="C108" s="3">
+      <c r="C108" s="51">
         <v>-1</v>
       </c>
       <c r="D108" s="3">
@@ -3883,7 +3883,7 @@
       <c r="B109" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="C109" s="3">
+      <c r="C109" s="51">
         <v>2</v>
       </c>
       <c r="D109" s="3">
@@ -3908,7 +3908,7 @@
       <c r="B110" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C110" s="3">
+      <c r="C110" s="51">
         <v>-1</v>
       </c>
       <c r="D110" s="3">
@@ -3932,7 +3932,7 @@
       <c r="B111" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C111" s="3">
+      <c r="C111" s="51">
         <v>1</v>
       </c>
       <c r="D111" s="3">
@@ -3955,7 +3955,7 @@
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="11"/>
       <c r="B112" s="15"/>
-      <c r="C112" s="3">
+      <c r="C112" s="51">
         <v>1</v>
       </c>
       <c r="D112" s="3">
@@ -4036,7 +4036,7 @@
       <c r="B116" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="C116" s="3">
+      <c r="C116" s="51">
         <v>1</v>
       </c>
       <c r="D116" s="3">
@@ -4059,7 +4059,7 @@
       <c r="B117" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C117" s="3">
+      <c r="C117" s="51">
         <v>1</v>
       </c>
       <c r="D117" s="3">
@@ -4085,7 +4085,7 @@
       <c r="B118" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="C118" s="3">
+      <c r="C118" s="51">
         <v>-2</v>
       </c>
       <c r="D118" s="3">
@@ -4107,7 +4107,7 @@
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="11"/>
       <c r="B119" s="15"/>
-      <c r="C119" s="3">
+      <c r="C119" s="51">
         <v>-1</v>
       </c>
       <c r="D119" s="3">
@@ -4131,7 +4131,7 @@
       <c r="B120" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C120" s="3">
+      <c r="C120" s="51">
         <v>-1</v>
       </c>
       <c r="D120" s="3">
@@ -4154,7 +4154,7 @@
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="11"/>
       <c r="B121" s="15"/>
-      <c r="C121" s="3">
+      <c r="C121" s="51">
         <v>-1</v>
       </c>
       <c r="D121" s="3">
@@ -4177,7 +4177,7 @@
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="11"/>
       <c r="B122" s="15"/>
-      <c r="C122" s="3">
+      <c r="C122" s="51">
         <v>-2</v>
       </c>
       <c r="D122" s="3">
@@ -4201,7 +4201,7 @@
       <c r="B123" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="C123" s="3">
+      <c r="C123" s="51">
         <v>2</v>
       </c>
       <c r="D123" s="3">
@@ -4226,7 +4226,7 @@
       <c r="B124" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C124" s="3">
+      <c r="C124" s="51">
         <v>-1</v>
       </c>
       <c r="D124" s="3">
@@ -4305,7 +4305,7 @@
       <c r="B128" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C128" s="3">
+      <c r="C128" s="51">
         <v>1</v>
       </c>
       <c r="D128" s="3">
@@ -4384,7 +4384,7 @@
       <c r="B132" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C132" s="3">
+      <c r="C132" s="51">
         <v>2</v>
       </c>
       <c r="D132" s="3">
@@ -4463,7 +4463,7 @@
       <c r="B136" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C136" s="3">
+      <c r="C136" s="51">
         <v>2</v>
       </c>
       <c r="D136" s="3">
@@ -4630,11 +4630,11 @@
       <c r="B145" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="C145" s="66">
+      <c r="C145" s="62">
         <f>J143</f>
         <v>1331142.8392085307</v>
       </c>
-      <c r="D145" s="67"/>
+      <c r="D145" s="63"/>
       <c r="E145" s="34"/>
       <c r="F145" s="36"/>
       <c r="G145" s="34"/>
@@ -4647,38 +4647,38 @@
       <c r="B146" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="C146" s="68">
+      <c r="C146" s="64">
         <f>0.13*C145</f>
         <v>173048.56909710899</v>
       </c>
-      <c r="D146" s="69"/>
+      <c r="D146" s="65"/>
     </row>
     <row r="147" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="40"/>
       <c r="B147" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="C147" s="68">
+      <c r="C147" s="64">
         <f>SUM(C145:D146)</f>
         <v>1504191.4083056396</v>
       </c>
-      <c r="D147" s="69"/>
+      <c r="D147" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="C145:D145"/>
     <mergeCell ref="C146:D146"/>
     <mergeCell ref="C147:D147"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>

</xml_diff>